<commit_message>
CI: één workflow voor GitHub Pages + optioneel Netlify en Cloudflare Pages
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/sterkteberekingen funderingswapening Romfix (1).xlsx
+++ b/sterkteberekingen funderingswapening Romfix (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3b3ce9f62cacfa1d/Romfix/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yenlo-my.sharepoint.com/personal/berntjan_bosma_yenlo_com/Documents/Bureaublad/Romfix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4343CC2F-9073-4518-94E3-F3DA523D61FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{4343CC2F-9073-4518-94E3-F3DA523D61FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{800AA4D0-F76F-4907-8B03-D252897EA3DD}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" tabRatio="791" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="791" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capping_Romfix" sheetId="115" r:id="rId1"/>
@@ -868,24 +868,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q151"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="3" width="13.19921875" style="16" customWidth="1"/>
-    <col min="4" max="4" width="13.06640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.19921875" style="16" customWidth="1"/>
-    <col min="6" max="6" width="13.19921875" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="11.796875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="11.19921875" style="15" customWidth="1"/>
-    <col min="10" max="10" width="10.796875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.796875" style="15" customWidth="1"/>
+    <col min="2" max="3" width="13.140625" style="16" customWidth="1"/>
+    <col min="4" max="4" width="13" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="16" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="15" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" style="15" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.85546875" style="15" customWidth="1"/>
     <col min="13" max="13" width="26" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.796875" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.73046875" style="16"/>
+    <col min="14" max="15" width="10.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>49</v>
       </c>
@@ -906,7 +906,7 @@
       <c r="P1" s="12"/>
       <c r="Q1" s="14"/>
     </row>
-    <row r="2" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
@@ -924,7 +924,7 @@
       <c r="P2" s="12"/>
       <c r="Q2" s="14"/>
     </row>
-    <row r="3" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>29</v>
       </c>
@@ -941,7 +941,7 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
@@ -956,7 +956,7 @@
       <c r="O4"/>
       <c r="P4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>30</v>
       </c>
@@ -977,7 +977,7 @@
       <c r="O5"/>
       <c r="P5"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
         <v>36</v>
       </c>
@@ -998,7 +998,7 @@
       <c r="O6"/>
       <c r="P6"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
         <v>37</v>
       </c>
@@ -1019,7 +1019,7 @@
       <c r="O7"/>
       <c r="P7"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>38</v>
       </c>
@@ -1040,7 +1040,7 @@
       <c r="O8"/>
       <c r="P8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
@@ -1055,7 +1055,7 @@
       <c r="O9"/>
       <c r="P9"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
         <v>32</v>
       </c>
@@ -1073,7 +1073,7 @@
       <c r="O10"/>
       <c r="P10"/>
     </row>
-    <row r="11" spans="1:17" ht="39.4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
         <v>20</v>
       </c>
@@ -1098,7 +1098,7 @@
       <c r="O11"/>
       <c r="P11"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>53</v>
       </c>
@@ -1129,7 +1129,7 @@
       <c r="O12"/>
       <c r="P12"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>55</v>
       </c>
@@ -1162,7 +1162,7 @@
       <c r="O13"/>
       <c r="P13"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>55</v>
       </c>
@@ -1191,7 +1191,7 @@
       <c r="O14"/>
       <c r="P14"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="17" t="s">
         <v>7</v>
       </c>
@@ -1222,7 +1222,7 @@
       <c r="O15"/>
       <c r="P15"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -1234,7 +1234,7 @@
       <c r="O16"/>
       <c r="P16"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
         <v>33</v>
       </c>
@@ -1252,7 +1252,7 @@
       <c r="O17"/>
       <c r="P17"/>
     </row>
-    <row r="18" spans="1:16" ht="39.4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
@@ -1277,7 +1277,7 @@
       <c r="O18"/>
       <c r="P18"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="17" t="str">
         <f>CONCATENATE("Wapening ",A13)</f>
         <v>Wapening Series 600 6F2 + R'cel + E'grid</v>
@@ -1304,7 +1304,7 @@
       <c r="O19"/>
       <c r="P19"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="str">
         <f>CONCATENATE("Wapening ",A14)</f>
         <v>Wapening Series 600 6F2 + R'cel + E'grid</v>
@@ -1331,7 +1331,7 @@
       <c r="O20"/>
       <c r="P20"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -1343,7 +1343,7 @@
       <c r="O21"/>
       <c r="P21"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
         <v>27</v>
       </c>
@@ -1362,7 +1362,7 @@
       <c r="O22"/>
       <c r="P22"/>
     </row>
-    <row r="23" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
         <v>20</v>
       </c>
@@ -1388,7 +1388,7 @@
       <c r="O23"/>
       <c r="P23"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="str">
         <f>A12</f>
         <v>Beton + fundering + series 800</v>
@@ -1418,7 +1418,7 @@
       <c r="O24"/>
       <c r="P24"/>
     </row>
-    <row r="25" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog</v>
@@ -1449,7 +1449,7 @@
       <c r="O25"/>
       <c r="P25"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend</v>
@@ -1477,7 +1477,7 @@
       <c r="O26"/>
       <c r="P26"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -1505,7 +1505,7 @@
       <c r="O27"/>
       <c r="P27"/>
     </row>
-    <row r="28" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog</v>
@@ -1536,7 +1536,7 @@
       <c r="O28"/>
       <c r="P28"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend</v>
@@ -1564,7 +1564,7 @@
       <c r="O29"/>
       <c r="P29"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -1592,7 +1592,7 @@
       <c r="O30"/>
       <c r="P30"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
         <v>7</v>
       </c>
@@ -1621,7 +1621,7 @@
       <c r="O31"/>
       <c r="P31"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -1636,7 +1636,7 @@
       <c r="O32"/>
       <c r="P32"/>
     </row>
-    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="18" t="s">
         <v>25</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="I33" s="29"/>
       <c r="J33" s="29"/>
     </row>
-    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="18" t="s">
         <v>3</v>
       </c>
@@ -1662,7 +1662,7 @@
       <c r="I34" s="29"/>
       <c r="J34" s="29"/>
     </row>
-    <row r="35" spans="1:16" s="31" customFormat="1" ht="52.5" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:16" s="31" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A35" s="19" t="s">
         <v>24</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="M35" s="30"/>
       <c r="N35" s="30"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" s="17" t="s">
         <v>23</v>
       </c>
@@ -1734,7 +1734,7 @@
       <c r="O36"/>
       <c r="P36"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" s="32" t="s">
         <v>16</v>
       </c>
@@ -1771,7 +1771,7 @@
       <c r="O37"/>
       <c r="P37"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" s="17" t="s">
         <v>21</v>
       </c>
@@ -1808,7 +1808,7 @@
       <c r="O38"/>
       <c r="P38"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" s="17" t="s">
         <v>22</v>
       </c>
@@ -1845,7 +1845,7 @@
       <c r="O39"/>
       <c r="P39"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" s="17" t="s">
         <v>2</v>
       </c>
@@ -1882,7 +1882,7 @@
       <c r="O40"/>
       <c r="P40"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" s="34" t="s">
         <v>11</v>
       </c>
@@ -1919,7 +1919,7 @@
       <c r="O41"/>
       <c r="P41"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="34" t="s">
         <v>12</v>
       </c>
@@ -1956,7 +1956,7 @@
       <c r="O42"/>
       <c r="P42"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" s="34" t="s">
         <v>13</v>
       </c>
@@ -1993,7 +1993,7 @@
       <c r="O43"/>
       <c r="P43"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="34" t="s">
         <v>14</v>
       </c>
@@ -2030,7 +2030,7 @@
       <c r="O44"/>
       <c r="P44"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" s="34" t="s">
         <v>15</v>
       </c>
@@ -2067,7 +2067,7 @@
       <c r="O45"/>
       <c r="P45"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="34" t="s">
         <v>10</v>
       </c>
@@ -2104,7 +2104,7 @@
       <c r="O46"/>
       <c r="P46"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="15"/>
@@ -2119,7 +2119,7 @@
       <c r="O47"/>
       <c r="P47"/>
     </row>
-    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="36" t="s">
         <v>26</v>
       </c>
@@ -2132,7 +2132,7 @@
       <c r="I48" s="29"/>
       <c r="J48" s="29"/>
     </row>
-    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="36" t="s">
         <v>46</v>
       </c>
@@ -2145,7 +2145,7 @@
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
     </row>
-    <row r="50" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" s="37" t="s">
         <v>20</v>
       </c>
@@ -2169,7 +2169,7 @@
       <c r="O50"/>
       <c r="P50"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2197,7 +2197,7 @@
       <c r="O51"/>
       <c r="P51"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2225,7 +2225,7 @@
       <c r="O52"/>
       <c r="P52"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2253,7 +2253,7 @@
       <c r="O53"/>
       <c r="P53"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2281,7 +2281,7 @@
       <c r="O54"/>
       <c r="P54"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2309,7 +2309,7 @@
       <c r="O55"/>
       <c r="P55"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2337,7 +2337,7 @@
       <c r="O56"/>
       <c r="P56"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
@@ -2352,7 +2352,7 @@
       <c r="O57"/>
       <c r="P57"/>
     </row>
-    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="18" t="s">
         <v>28</v>
       </c>
@@ -2365,7 +2365,7 @@
       <c r="I58" s="29"/>
       <c r="J58" s="29"/>
     </row>
-    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="18" t="s">
         <v>31</v>
       </c>
@@ -2378,7 +2378,7 @@
       <c r="I59" s="29"/>
       <c r="J59" s="29"/>
     </row>
-    <row r="60" spans="1:16" s="31" customFormat="1" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:16" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="19" t="s">
         <v>20</v>
       </c>
@@ -2401,7 +2401,7 @@
       <c r="J60" s="30"/>
       <c r="K60" s="30"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2433,7 +2433,7 @@
       <c r="O61"/>
       <c r="P61"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2465,7 +2465,7 @@
       <c r="O62"/>
       <c r="P62"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2497,7 +2497,7 @@
       <c r="O63"/>
       <c r="P63"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2529,7 +2529,7 @@
       <c r="O64"/>
       <c r="P64"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2561,7 +2561,7 @@
       <c r="O65"/>
       <c r="P65"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2593,7 +2593,7 @@
       <c r="O66"/>
       <c r="P66"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" s="17" t="str">
         <f>CONCATENATE(A$14," volledig ongewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid volledig ongewapend en dieper</v>
@@ -2625,7 +2625,7 @@
       <c r="O67"/>
       <c r="P67"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="15"/>
@@ -2640,7 +2640,7 @@
       <c r="O68"/>
       <c r="P68"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="15"/>
@@ -2655,7 +2655,7 @@
       <c r="O69"/>
       <c r="P69"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="15"/>
@@ -2670,7 +2670,7 @@
       <c r="O70"/>
       <c r="P70"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="15"/>
@@ -2685,7 +2685,7 @@
       <c r="O71"/>
       <c r="P71"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="15"/>
@@ -2700,7 +2700,7 @@
       <c r="O72"/>
       <c r="P72"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="15"/>
@@ -2715,7 +2715,7 @@
       <c r="O73"/>
       <c r="P73"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="15"/>
@@ -2730,7 +2730,7 @@
       <c r="O74"/>
       <c r="P74"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="15"/>
@@ -2745,7 +2745,7 @@
       <c r="O75"/>
       <c r="P75"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="15"/>
@@ -2760,7 +2760,7 @@
       <c r="O76"/>
       <c r="P76"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="15"/>
@@ -2775,7 +2775,7 @@
       <c r="O77"/>
       <c r="P77"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="15"/>
@@ -2790,7 +2790,7 @@
       <c r="O78"/>
       <c r="P78"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="15"/>
@@ -2805,7 +2805,7 @@
       <c r="O79"/>
       <c r="P79"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="15"/>
@@ -2820,7 +2820,7 @@
       <c r="O80"/>
       <c r="P80"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="15"/>
@@ -2835,7 +2835,7 @@
       <c r="O81"/>
       <c r="P81"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="15"/>
@@ -2850,7 +2850,7 @@
       <c r="O82"/>
       <c r="P82"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="15"/>
@@ -2865,7 +2865,7 @@
       <c r="O83"/>
       <c r="P83"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="15"/>
@@ -2880,7 +2880,7 @@
       <c r="O84"/>
       <c r="P84"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="15"/>
@@ -2895,7 +2895,7 @@
       <c r="O85"/>
       <c r="P85"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="15"/>
@@ -2910,7 +2910,7 @@
       <c r="O86"/>
       <c r="P86"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="15"/>
@@ -2925,7 +2925,7 @@
       <c r="O87"/>
       <c r="P87"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="15"/>
@@ -2940,7 +2940,7 @@
       <c r="O88"/>
       <c r="P88"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
@@ -2955,7 +2955,7 @@
       <c r="O89"/>
       <c r="P89"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="15"/>
@@ -2970,7 +2970,7 @@
       <c r="O90"/>
       <c r="P90"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="15"/>
@@ -2985,7 +2985,7 @@
       <c r="O91"/>
       <c r="P91"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="15"/>
@@ -3000,7 +3000,7 @@
       <c r="O92"/>
       <c r="P92"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="15"/>
@@ -3015,7 +3015,7 @@
       <c r="O93"/>
       <c r="P93"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="15"/>
@@ -3030,7 +3030,7 @@
       <c r="O94"/>
       <c r="P94"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="15"/>
@@ -3045,7 +3045,7 @@
       <c r="O95"/>
       <c r="P95"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="15"/>
@@ -3060,7 +3060,7 @@
       <c r="O96"/>
       <c r="P96"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -3075,7 +3075,7 @@
       <c r="O97"/>
       <c r="P97"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -3090,7 +3090,7 @@
       <c r="O98"/>
       <c r="P98"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -3105,7 +3105,7 @@
       <c r="O99"/>
       <c r="P99"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="15"/>
@@ -3120,7 +3120,7 @@
       <c r="O100"/>
       <c r="P100"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="15"/>
@@ -3135,7 +3135,7 @@
       <c r="O101"/>
       <c r="P101"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="15"/>
@@ -3150,7 +3150,7 @@
       <c r="O102"/>
       <c r="P102"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="15"/>
@@ -3165,7 +3165,7 @@
       <c r="O103"/>
       <c r="P103"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="15"/>
@@ -3180,7 +3180,7 @@
       <c r="O104"/>
       <c r="P104"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="15"/>
@@ -3195,7 +3195,7 @@
       <c r="O105"/>
       <c r="P105"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="15"/>
@@ -3210,7 +3210,7 @@
       <c r="O106"/>
       <c r="P106"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="15"/>
@@ -3225,7 +3225,7 @@
       <c r="O107"/>
       <c r="P107"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="15"/>
@@ -3240,7 +3240,7 @@
       <c r="O108"/>
       <c r="P108"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="15"/>
@@ -3255,7 +3255,7 @@
       <c r="O109"/>
       <c r="P109"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="15"/>
@@ -3270,7 +3270,7 @@
       <c r="O110"/>
       <c r="P110"/>
     </row>
-    <row r="111" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="15"/>
@@ -3285,7 +3285,7 @@
       <c r="O111"/>
       <c r="P111"/>
     </row>
-    <row r="112" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3300,7 +3300,7 @@
       <c r="O112"/>
       <c r="P112"/>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3315,7 +3315,7 @@
       <c r="O113"/>
       <c r="P113"/>
     </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -3330,7 +3330,7 @@
       <c r="O114"/>
       <c r="P114"/>
     </row>
-    <row r="115" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -3345,7 +3345,7 @@
       <c r="O115"/>
       <c r="P115"/>
     </row>
-    <row r="116" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -3360,7 +3360,7 @@
       <c r="O116"/>
       <c r="P116"/>
     </row>
-    <row r="117" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="15"/>
@@ -3375,7 +3375,7 @@
       <c r="O117"/>
       <c r="P117"/>
     </row>
-    <row r="118" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="15"/>
@@ -3390,7 +3390,7 @@
       <c r="O118"/>
       <c r="P118"/>
     </row>
-    <row r="119" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="15"/>
@@ -3405,7 +3405,7 @@
       <c r="O119"/>
       <c r="P119"/>
     </row>
-    <row r="120" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="15"/>
@@ -3420,7 +3420,7 @@
       <c r="O120"/>
       <c r="P120"/>
     </row>
-    <row r="121" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="15"/>
@@ -3435,7 +3435,7 @@
       <c r="O121"/>
       <c r="P121"/>
     </row>
-    <row r="122" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="15"/>
@@ -3450,7 +3450,7 @@
       <c r="O122"/>
       <c r="P122"/>
     </row>
-    <row r="123" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="15"/>
@@ -3465,7 +3465,7 @@
       <c r="O123"/>
       <c r="P123"/>
     </row>
-    <row r="124" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="15"/>
@@ -3480,7 +3480,7 @@
       <c r="O124"/>
       <c r="P124"/>
     </row>
-    <row r="125" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
@@ -3495,7 +3495,7 @@
       <c r="O125"/>
       <c r="P125"/>
     </row>
-    <row r="126" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -3510,7 +3510,7 @@
       <c r="O126"/>
       <c r="P126"/>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3525,7 +3525,7 @@
       <c r="O127"/>
       <c r="P127"/>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3540,7 +3540,7 @@
       <c r="O128"/>
       <c r="P128"/>
     </row>
-    <row r="129" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -3555,7 +3555,7 @@
       <c r="O129"/>
       <c r="P129"/>
     </row>
-    <row r="130" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -3570,7 +3570,7 @@
       <c r="O130"/>
       <c r="P130"/>
     </row>
-    <row r="131" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
@@ -3585,7 +3585,7 @@
       <c r="O131"/>
       <c r="P131"/>
     </row>
-    <row r="132" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="15"/>
@@ -3600,7 +3600,7 @@
       <c r="O132"/>
       <c r="P132"/>
     </row>
-    <row r="133" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="15"/>
@@ -3615,7 +3615,7 @@
       <c r="O133"/>
       <c r="P133"/>
     </row>
-    <row r="134" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="15"/>
@@ -3630,7 +3630,7 @@
       <c r="O134"/>
       <c r="P134"/>
     </row>
-    <row r="135" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="15"/>
@@ -3645,7 +3645,7 @@
       <c r="O135"/>
       <c r="P135"/>
     </row>
-    <row r="136" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="15"/>
@@ -3660,7 +3660,7 @@
       <c r="O136"/>
       <c r="P136"/>
     </row>
-    <row r="137" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="15"/>
@@ -3675,7 +3675,7 @@
       <c r="O137"/>
       <c r="P137"/>
     </row>
-    <row r="138" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -3690,7 +3690,7 @@
       <c r="O138"/>
       <c r="P138"/>
     </row>
-    <row r="139" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -3705,7 +3705,7 @@
       <c r="O139"/>
       <c r="P139"/>
     </row>
-    <row r="140" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
@@ -3720,7 +3720,7 @@
       <c r="O140"/>
       <c r="P140"/>
     </row>
-    <row r="141" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -3735,7 +3735,7 @@
       <c r="O141"/>
       <c r="P141"/>
     </row>
-    <row r="142" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -3750,7 +3750,7 @@
       <c r="O142"/>
       <c r="P142"/>
     </row>
-    <row r="143" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -3765,7 +3765,7 @@
       <c r="O143"/>
       <c r="P143"/>
     </row>
-    <row r="144" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -3780,7 +3780,7 @@
       <c r="O144"/>
       <c r="P144"/>
     </row>
-    <row r="145" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
@@ -3795,7 +3795,7 @@
       <c r="O145"/>
       <c r="P145"/>
     </row>
-    <row r="146" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="15"/>
@@ -3810,7 +3810,7 @@
       <c r="O146"/>
       <c r="P146"/>
     </row>
-    <row r="147" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="15"/>
@@ -3825,7 +3825,7 @@
       <c r="O147"/>
       <c r="P147"/>
     </row>
-    <row r="148" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="148" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="15"/>
@@ -3840,7 +3840,7 @@
       <c r="O148"/>
       <c r="P148"/>
     </row>
-    <row r="149" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="15"/>
@@ -3855,7 +3855,7 @@
       <c r="O149"/>
       <c r="P149"/>
     </row>
-    <row r="150" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="150" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="15"/>
@@ -3870,7 +3870,7 @@
       <c r="O150"/>
       <c r="P150"/>
     </row>
-    <row r="151" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="151" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="15"/>
@@ -3917,24 +3917,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q151"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="44.06640625" customWidth="1"/>
-    <col min="2" max="3" width="13.19921875" style="16" customWidth="1"/>
-    <col min="4" max="4" width="13.06640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.19921875" style="16" customWidth="1"/>
-    <col min="6" max="6" width="13.19921875" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="11.796875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="11.19921875" style="15" customWidth="1"/>
-    <col min="10" max="10" width="10.796875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.796875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="3" width="13.140625" style="16" customWidth="1"/>
+    <col min="4" max="4" width="13" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="16" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="15" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" style="15" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.85546875" style="15" customWidth="1"/>
     <col min="13" max="13" width="26" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.796875" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.73046875" style="16"/>
+    <col min="14" max="15" width="10.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>49</v>
       </c>
@@ -3955,7 +3955,7 @@
       <c r="P1" s="12"/>
       <c r="Q1" s="14"/>
     </row>
-    <row r="2" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
@@ -3973,7 +3973,7 @@
       <c r="P2" s="12"/>
       <c r="Q2" s="14"/>
     </row>
-    <row r="3" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>29</v>
       </c>
@@ -3990,7 +3990,7 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
@@ -4005,7 +4005,7 @@
       <c r="O4"/>
       <c r="P4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>30</v>
       </c>
@@ -4026,7 +4026,7 @@
       <c r="O5"/>
       <c r="P5"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
         <v>36</v>
       </c>
@@ -4047,7 +4047,7 @@
       <c r="O6"/>
       <c r="P6"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
         <v>37</v>
       </c>
@@ -4068,7 +4068,7 @@
       <c r="O7"/>
       <c r="P7"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>38</v>
       </c>
@@ -4089,7 +4089,7 @@
       <c r="O8"/>
       <c r="P8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
@@ -4104,7 +4104,7 @@
       <c r="O9"/>
       <c r="P9"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
         <v>32</v>
       </c>
@@ -4122,7 +4122,7 @@
       <c r="O10"/>
       <c r="P10"/>
     </row>
-    <row r="11" spans="1:17" ht="39.4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
         <v>20</v>
       </c>
@@ -4147,7 +4147,7 @@
       <c r="O11"/>
       <c r="P11"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>52</v>
       </c>
@@ -4178,7 +4178,7 @@
       <c r="O12"/>
       <c r="P12"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -4186,15 +4186,15 @@
         <v>250</v>
       </c>
       <c r="C13" s="2">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="D13" s="9">
         <f>IF(F13="vast",C13,IF(F13="vrij",G46,""))</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E13" s="5">
         <f>IF(F13="vrij",E25,IF(F13="vast",MAX(D13,E25),""))</f>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>51</v>
@@ -4211,7 +4211,7 @@
       <c r="O13"/>
       <c r="P13"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>56</v>
       </c>
@@ -4240,7 +4240,7 @@
       <c r="O14"/>
       <c r="P14"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="17" t="s">
         <v>7</v>
       </c>
@@ -4271,7 +4271,7 @@
       <c r="O15"/>
       <c r="P15"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -4283,7 +4283,7 @@
       <c r="O16"/>
       <c r="P16"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="18" t="s">
         <v>33</v>
       </c>
@@ -4301,7 +4301,7 @@
       <c r="O17"/>
       <c r="P17"/>
     </row>
-    <row r="18" spans="1:16" ht="39.4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
@@ -4326,7 +4326,7 @@
       <c r="O18"/>
       <c r="P18"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="17" t="str">
         <f>CONCATENATE("Wapening ",A13)</f>
         <v>Wapening Series 800 Type 1 + R'cel + E'grid</v>
@@ -4353,7 +4353,7 @@
       <c r="O19"/>
       <c r="P19"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="str">
         <f>CONCATENATE("Wapening ",A14)</f>
         <v>Wapening Series 800 Type 1 + R'cel + E'grid</v>
@@ -4380,7 +4380,7 @@
       <c r="O20"/>
       <c r="P20"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -4392,7 +4392,7 @@
       <c r="O21"/>
       <c r="P21"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="18" t="s">
         <v>27</v>
       </c>
@@ -4411,7 +4411,7 @@
       <c r="O22"/>
       <c r="P22"/>
     </row>
-    <row r="23" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
         <v>20</v>
       </c>
@@ -4437,7 +4437,7 @@
       <c r="O23"/>
       <c r="P23"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="str">
         <f>A12</f>
         <v>Beton + fundering</v>
@@ -4467,7 +4467,7 @@
       <c r="O24"/>
       <c r="P24"/>
     </row>
-    <row r="25" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog</v>
@@ -4482,11 +4482,11 @@
       </c>
       <c r="D25" s="22">
         <f>IF(B25=0,D26,ROUND(D28/F61,0))</f>
-        <v>381</v>
+        <v>282</v>
       </c>
       <c r="E25" s="23">
         <f>D51</f>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="F25" s="24"/>
       <c r="H25"/>
@@ -4498,7 +4498,7 @@
       <c r="O25"/>
       <c r="P25"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend</v>
@@ -4509,11 +4509,11 @@
       </c>
       <c r="C26" s="5">
         <f>IF(B26=0,0,ROUND(MIN(D19*D27,E19*C13),0))</f>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="D26" s="5">
         <f>IF(B26=0,D27,ROUND(D28/F62,0))</f>
-        <v>381</v>
+        <v>282</v>
       </c>
       <c r="E26" s="25"/>
       <c r="F26" s="24"/>
@@ -4526,7 +4526,7 @@
       <c r="O26"/>
       <c r="P26"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -4554,7 +4554,7 @@
       <c r="O27"/>
       <c r="P27"/>
     </row>
-    <row r="28" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog</v>
@@ -4585,7 +4585,7 @@
       <c r="O28"/>
       <c r="P28"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend</v>
@@ -4613,7 +4613,7 @@
       <c r="O29"/>
       <c r="P29"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -4641,7 +4641,7 @@
       <c r="O30"/>
       <c r="P30"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="17" t="s">
         <v>7</v>
       </c>
@@ -4670,7 +4670,7 @@
       <c r="O31"/>
       <c r="P31"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -4685,7 +4685,7 @@
       <c r="O32"/>
       <c r="P32"/>
     </row>
-    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="18" t="s">
         <v>25</v>
       </c>
@@ -4698,7 +4698,7 @@
       <c r="I33" s="29"/>
       <c r="J33" s="29"/>
     </row>
-    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="18" t="s">
         <v>3</v>
       </c>
@@ -4711,7 +4711,7 @@
       <c r="I34" s="29"/>
       <c r="J34" s="29"/>
     </row>
-    <row r="35" spans="1:16" s="31" customFormat="1" ht="52.5" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:16" s="31" customFormat="1" ht="51" x14ac:dyDescent="0.2">
       <c r="A35" s="19" t="s">
         <v>24</v>
       </c>
@@ -4746,7 +4746,7 @@
       <c r="M35" s="30"/>
       <c r="N35" s="30"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" s="17" t="s">
         <v>23</v>
       </c>
@@ -4783,7 +4783,7 @@
       <c r="O36"/>
       <c r="P36"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" s="32" t="s">
         <v>16</v>
       </c>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="E37" s="23">
         <f>D26</f>
-        <v>381</v>
+        <v>282</v>
       </c>
       <c r="F37" s="5">
         <f>C15</f>
@@ -4820,7 +4820,7 @@
       <c r="O37"/>
       <c r="P37"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" s="17" t="s">
         <v>21</v>
       </c>
@@ -4834,11 +4834,11 @@
       </c>
       <c r="D38" s="5">
         <f>C13</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E38" s="5">
         <f>C13</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F38" s="5">
         <f>C14</f>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="G38" s="5">
         <f>C13</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H38" s="16"/>
       <c r="I38" s="16"/>
@@ -4857,7 +4857,7 @@
       <c r="O38"/>
       <c r="P38"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" s="17" t="s">
         <v>22</v>
       </c>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="E39" s="6">
         <f t="shared" si="0"/>
-        <v>381</v>
+        <v>282</v>
       </c>
       <c r="F39" s="6">
         <f t="shared" si="0"/>
@@ -4894,7 +4894,7 @@
       <c r="O39"/>
       <c r="P39"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" s="17" t="s">
         <v>2</v>
       </c>
@@ -4931,7 +4931,7 @@
       <c r="O40"/>
       <c r="P40"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" s="34" t="s">
         <v>11</v>
       </c>
@@ -4945,11 +4945,11 @@
       </c>
       <c r="D41" s="35">
         <f t="shared" si="2"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E41" s="35">
         <f t="shared" si="2"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F41" s="35">
         <f t="shared" si="2"/>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="G41" s="35">
         <f t="shared" si="2"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H41" s="16"/>
       <c r="I41" s="16"/>
@@ -4968,7 +4968,7 @@
       <c r="O41"/>
       <c r="P41"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" s="34" t="s">
         <v>12</v>
       </c>
@@ -4982,11 +4982,11 @@
       </c>
       <c r="D42" s="35">
         <f t="shared" si="3"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E42" s="35">
         <f t="shared" si="3"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F42" s="35">
         <f t="shared" si="3"/>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="G42" s="35">
         <f t="shared" si="3"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H42" s="16"/>
       <c r="I42" s="16"/>
@@ -5005,7 +5005,7 @@
       <c r="O42"/>
       <c r="P42"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" s="34" t="s">
         <v>13</v>
       </c>
@@ -5019,11 +5019,11 @@
       </c>
       <c r="D43" s="35">
         <f t="shared" si="4"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E43" s="35">
         <f t="shared" si="4"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F43" s="35">
         <f t="shared" si="4"/>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="G43" s="35">
         <f t="shared" si="4"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H43" s="16"/>
       <c r="I43" s="16"/>
@@ -5042,7 +5042,7 @@
       <c r="O43"/>
       <c r="P43"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" s="34" t="s">
         <v>14</v>
       </c>
@@ -5056,11 +5056,11 @@
       </c>
       <c r="D44" s="35">
         <f t="shared" si="5"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E44" s="35">
         <f t="shared" si="5"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F44" s="35">
         <f t="shared" si="5"/>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="G44" s="35">
         <f t="shared" si="5"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H44" s="16"/>
       <c r="I44" s="16"/>
@@ -5079,7 +5079,7 @@
       <c r="O44"/>
       <c r="P44"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" s="34" t="s">
         <v>15</v>
       </c>
@@ -5093,11 +5093,11 @@
       </c>
       <c r="D45" s="35">
         <f t="shared" ref="D45:E45" si="6">MIN(D40*D37,D38)</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E45" s="35">
         <f t="shared" si="6"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F45" s="35">
         <f>MIN(F40*F37,F38)</f>
@@ -5105,7 +5105,7 @@
       </c>
       <c r="G45" s="35">
         <f>MIN(G40*G37,G38)</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H45" s="16"/>
       <c r="I45" s="16"/>
@@ -5116,7 +5116,7 @@
       <c r="O45"/>
       <c r="P45"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" s="34" t="s">
         <v>10</v>
       </c>
@@ -5130,11 +5130,11 @@
       </c>
       <c r="D46" s="35">
         <f t="shared" si="7"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="E46" s="35">
         <f t="shared" si="7"/>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="F46" s="35">
         <f>ROUND(AVERAGE(F41:F45),0)</f>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="G46" s="35">
         <f>ROUND(AVERAGE(G41:G45),0)</f>
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="H46" s="16"/>
       <c r="I46" s="16"/>
@@ -5153,7 +5153,7 @@
       <c r="O46"/>
       <c r="P46"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="15"/>
@@ -5168,7 +5168,7 @@
       <c r="O47"/>
       <c r="P47"/>
     </row>
-    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="36" t="s">
         <v>26</v>
       </c>
@@ -5181,7 +5181,7 @@
       <c r="I48" s="29"/>
       <c r="J48" s="29"/>
     </row>
-    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="36" t="s">
         <v>46</v>
       </c>
@@ -5194,7 +5194,7 @@
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
     </row>
-    <row r="50" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" s="37" t="s">
         <v>20</v>
       </c>
@@ -5218,7 +5218,7 @@
       <c r="O50"/>
       <c r="P50"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="D51" s="5">
         <f>ROUND(((B51*C51^(1/3)+B52*C52^(1/3)+B53*C53^(1/3))/(B51+B52+B53))^3,0)</f>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="E51" s="15"/>
       <c r="F51" s="15"/>
@@ -5246,7 +5246,7 @@
       <c r="O51"/>
       <c r="P51"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5257,11 +5257,11 @@
       </c>
       <c r="C52" s="38">
         <f t="shared" si="9"/>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="D52" s="5">
         <f>IF(B52+B53=0,0,IF(B53=0,C52,ROUND(((B52*C52^(1/3)+B53*C53^(1/3))/(B52+B53))^3,0)))</f>
-        <v>645</v>
+        <v>344</v>
       </c>
       <c r="E52" s="15"/>
       <c r="F52" s="15"/>
@@ -5274,7 +5274,7 @@
       <c r="O52"/>
       <c r="P52"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5302,7 +5302,7 @@
       <c r="O53"/>
       <c r="P53"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5330,7 +5330,7 @@
       <c r="O54"/>
       <c r="P54"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5358,7 +5358,7 @@
       <c r="O55"/>
       <c r="P55"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5386,7 +5386,7 @@
       <c r="O56"/>
       <c r="P56"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
@@ -5401,7 +5401,7 @@
       <c r="O57"/>
       <c r="P57"/>
     </row>
-    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="18" t="s">
         <v>28</v>
       </c>
@@ -5414,7 +5414,7 @@
       <c r="I58" s="29"/>
       <c r="J58" s="29"/>
     </row>
-    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="18" t="s">
         <v>31</v>
       </c>
@@ -5427,7 +5427,7 @@
       <c r="I59" s="29"/>
       <c r="J59" s="29"/>
     </row>
-    <row r="60" spans="1:16" s="31" customFormat="1" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:16" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="19" t="s">
         <v>20</v>
       </c>
@@ -5450,7 +5450,7 @@
       <c r="J60" s="30"/>
       <c r="K60" s="30"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5468,11 +5468,11 @@
       </c>
       <c r="E61" s="40">
         <f>D51/D28</f>
-        <v>2.7564102564102564</v>
+        <v>1.4700854700854702</v>
       </c>
       <c r="F61" s="40">
         <f>IF(D61="","",(B61/SQRT(B61^2+C61^2*E61^(2/3)))*(1-1/E61)+1/E61)</f>
-        <v>0.61348089534453298</v>
+        <v>0.82946507354766585</v>
       </c>
       <c r="H61"/>
       <c r="J61" s="16"/>
@@ -5482,7 +5482,7 @@
       <c r="O61"/>
       <c r="P61"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5500,11 +5500,11 @@
       </c>
       <c r="E62" s="40">
         <f>D52/D28</f>
-        <v>2.7564102564102564</v>
+        <v>1.4700854700854702</v>
       </c>
       <c r="F62" s="40">
         <f t="shared" ref="F62:F67" si="11">IF(D62="","",(B62/SQRT(B62^2+C62^2*E62^(2/3)))*(1-1/E62)+1/E62)</f>
-        <v>0.61348089534453298</v>
+        <v>0.82946507354766585</v>
       </c>
       <c r="H62"/>
       <c r="J62" s="16"/>
@@ -5514,7 +5514,7 @@
       <c r="O62"/>
       <c r="P62"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5546,7 +5546,7 @@
       <c r="O63"/>
       <c r="P63"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5578,7 +5578,7 @@
       <c r="O64"/>
       <c r="P64"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5610,7 +5610,7 @@
       <c r="O65"/>
       <c r="P65"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5642,7 +5642,7 @@
       <c r="O66"/>
       <c r="P66"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" s="17" t="str">
         <f>CONCATENATE(A$14," volledig ongewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid volledig ongewapend en dieper</v>
@@ -5674,7 +5674,7 @@
       <c r="O67"/>
       <c r="P67"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="15"/>
@@ -5689,7 +5689,7 @@
       <c r="O68"/>
       <c r="P68"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="15"/>
@@ -5704,7 +5704,7 @@
       <c r="O69"/>
       <c r="P69"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="15"/>
@@ -5719,7 +5719,7 @@
       <c r="O70"/>
       <c r="P70"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="15"/>
@@ -5734,7 +5734,7 @@
       <c r="O71"/>
       <c r="P71"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="15"/>
@@ -5749,7 +5749,7 @@
       <c r="O72"/>
       <c r="P72"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="15"/>
@@ -5764,7 +5764,7 @@
       <c r="O73"/>
       <c r="P73"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="15"/>
@@ -5779,7 +5779,7 @@
       <c r="O74"/>
       <c r="P74"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="15"/>
@@ -5794,7 +5794,7 @@
       <c r="O75"/>
       <c r="P75"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="15"/>
@@ -5809,7 +5809,7 @@
       <c r="O76"/>
       <c r="P76"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="15"/>
@@ -5824,7 +5824,7 @@
       <c r="O77"/>
       <c r="P77"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="15"/>
@@ -5839,7 +5839,7 @@
       <c r="O78"/>
       <c r="P78"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="15"/>
@@ -5854,7 +5854,7 @@
       <c r="O79"/>
       <c r="P79"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="15"/>
@@ -5869,7 +5869,7 @@
       <c r="O80"/>
       <c r="P80"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="15"/>
@@ -5884,7 +5884,7 @@
       <c r="O81"/>
       <c r="P81"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="15"/>
@@ -5899,7 +5899,7 @@
       <c r="O82"/>
       <c r="P82"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="15"/>
@@ -5914,7 +5914,7 @@
       <c r="O83"/>
       <c r="P83"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="15"/>
@@ -5929,7 +5929,7 @@
       <c r="O84"/>
       <c r="P84"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="15"/>
@@ -5944,7 +5944,7 @@
       <c r="O85"/>
       <c r="P85"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="15"/>
@@ -5959,7 +5959,7 @@
       <c r="O86"/>
       <c r="P86"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="15"/>
@@ -5974,7 +5974,7 @@
       <c r="O87"/>
       <c r="P87"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="15"/>
@@ -5989,7 +5989,7 @@
       <c r="O88"/>
       <c r="P88"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
@@ -6004,7 +6004,7 @@
       <c r="O89"/>
       <c r="P89"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="15"/>
@@ -6019,7 +6019,7 @@
       <c r="O90"/>
       <c r="P90"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="15"/>
@@ -6034,7 +6034,7 @@
       <c r="O91"/>
       <c r="P91"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="15"/>
@@ -6049,7 +6049,7 @@
       <c r="O92"/>
       <c r="P92"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="15"/>
@@ -6064,7 +6064,7 @@
       <c r="O93"/>
       <c r="P93"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="15"/>
@@ -6079,7 +6079,7 @@
       <c r="O94"/>
       <c r="P94"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="15"/>
@@ -6094,7 +6094,7 @@
       <c r="O95"/>
       <c r="P95"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="15"/>
@@ -6109,7 +6109,7 @@
       <c r="O96"/>
       <c r="P96"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -6124,7 +6124,7 @@
       <c r="O97"/>
       <c r="P97"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -6139,7 +6139,7 @@
       <c r="O98"/>
       <c r="P98"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -6154,7 +6154,7 @@
       <c r="O99"/>
       <c r="P99"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="15"/>
@@ -6169,7 +6169,7 @@
       <c r="O100"/>
       <c r="P100"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="15"/>
@@ -6184,7 +6184,7 @@
       <c r="O101"/>
       <c r="P101"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="15"/>
@@ -6199,7 +6199,7 @@
       <c r="O102"/>
       <c r="P102"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="15"/>
@@ -6214,7 +6214,7 @@
       <c r="O103"/>
       <c r="P103"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="15"/>
@@ -6229,7 +6229,7 @@
       <c r="O104"/>
       <c r="P104"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="15"/>
@@ -6244,7 +6244,7 @@
       <c r="O105"/>
       <c r="P105"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="15"/>
@@ -6259,7 +6259,7 @@
       <c r="O106"/>
       <c r="P106"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="15"/>
@@ -6274,7 +6274,7 @@
       <c r="O107"/>
       <c r="P107"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="15"/>
@@ -6289,7 +6289,7 @@
       <c r="O108"/>
       <c r="P108"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="15"/>
@@ -6304,7 +6304,7 @@
       <c r="O109"/>
       <c r="P109"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="15"/>
@@ -6319,7 +6319,7 @@
       <c r="O110"/>
       <c r="P110"/>
     </row>
-    <row r="111" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="15"/>
@@ -6334,7 +6334,7 @@
       <c r="O111"/>
       <c r="P111"/>
     </row>
-    <row r="112" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -6349,7 +6349,7 @@
       <c r="O112"/>
       <c r="P112"/>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -6364,7 +6364,7 @@
       <c r="O113"/>
       <c r="P113"/>
     </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -6379,7 +6379,7 @@
       <c r="O114"/>
       <c r="P114"/>
     </row>
-    <row r="115" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -6394,7 +6394,7 @@
       <c r="O115"/>
       <c r="P115"/>
     </row>
-    <row r="116" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -6409,7 +6409,7 @@
       <c r="O116"/>
       <c r="P116"/>
     </row>
-    <row r="117" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="15"/>
@@ -6424,7 +6424,7 @@
       <c r="O117"/>
       <c r="P117"/>
     </row>
-    <row r="118" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="15"/>
@@ -6439,7 +6439,7 @@
       <c r="O118"/>
       <c r="P118"/>
     </row>
-    <row r="119" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="15"/>
@@ -6454,7 +6454,7 @@
       <c r="O119"/>
       <c r="P119"/>
     </row>
-    <row r="120" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="15"/>
@@ -6469,7 +6469,7 @@
       <c r="O120"/>
       <c r="P120"/>
     </row>
-    <row r="121" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="15"/>
@@ -6484,7 +6484,7 @@
       <c r="O121"/>
       <c r="P121"/>
     </row>
-    <row r="122" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="15"/>
@@ -6499,7 +6499,7 @@
       <c r="O122"/>
       <c r="P122"/>
     </row>
-    <row r="123" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="15"/>
@@ -6514,7 +6514,7 @@
       <c r="O123"/>
       <c r="P123"/>
     </row>
-    <row r="124" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="15"/>
@@ -6529,7 +6529,7 @@
       <c r="O124"/>
       <c r="P124"/>
     </row>
-    <row r="125" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
@@ -6544,7 +6544,7 @@
       <c r="O125"/>
       <c r="P125"/>
     </row>
-    <row r="126" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -6559,7 +6559,7 @@
       <c r="O126"/>
       <c r="P126"/>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -6574,7 +6574,7 @@
       <c r="O127"/>
       <c r="P127"/>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -6589,7 +6589,7 @@
       <c r="O128"/>
       <c r="P128"/>
     </row>
-    <row r="129" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -6604,7 +6604,7 @@
       <c r="O129"/>
       <c r="P129"/>
     </row>
-    <row r="130" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="130" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -6619,7 +6619,7 @@
       <c r="O130"/>
       <c r="P130"/>
     </row>
-    <row r="131" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
@@ -6634,7 +6634,7 @@
       <c r="O131"/>
       <c r="P131"/>
     </row>
-    <row r="132" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="15"/>
@@ -6649,7 +6649,7 @@
       <c r="O132"/>
       <c r="P132"/>
     </row>
-    <row r="133" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="15"/>
@@ -6664,7 +6664,7 @@
       <c r="O133"/>
       <c r="P133"/>
     </row>
-    <row r="134" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="15"/>
@@ -6679,7 +6679,7 @@
       <c r="O134"/>
       <c r="P134"/>
     </row>
-    <row r="135" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="15"/>
@@ -6694,7 +6694,7 @@
       <c r="O135"/>
       <c r="P135"/>
     </row>
-    <row r="136" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="136" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="15"/>
@@ -6709,7 +6709,7 @@
       <c r="O136"/>
       <c r="P136"/>
     </row>
-    <row r="137" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="15"/>
@@ -6724,7 +6724,7 @@
       <c r="O137"/>
       <c r="P137"/>
     </row>
-    <row r="138" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -6739,7 +6739,7 @@
       <c r="O138"/>
       <c r="P138"/>
     </row>
-    <row r="139" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -6754,7 +6754,7 @@
       <c r="O139"/>
       <c r="P139"/>
     </row>
-    <row r="140" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
@@ -6769,7 +6769,7 @@
       <c r="O140"/>
       <c r="P140"/>
     </row>
-    <row r="141" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="141" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -6784,7 +6784,7 @@
       <c r="O141"/>
       <c r="P141"/>
     </row>
-    <row r="142" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -6799,7 +6799,7 @@
       <c r="O142"/>
       <c r="P142"/>
     </row>
-    <row r="143" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -6814,7 +6814,7 @@
       <c r="O143"/>
       <c r="P143"/>
     </row>
-    <row r="144" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -6829,7 +6829,7 @@
       <c r="O144"/>
       <c r="P144"/>
     </row>
-    <row r="145" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
@@ -6844,7 +6844,7 @@
       <c r="O145"/>
       <c r="P145"/>
     </row>
-    <row r="146" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="15"/>
@@ -6859,7 +6859,7 @@
       <c r="O146"/>
       <c r="P146"/>
     </row>
-    <row r="147" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="15"/>
@@ -6874,7 +6874,7 @@
       <c r="O147"/>
       <c r="P147"/>
     </row>
-    <row r="148" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="148" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="15"/>
@@ -6889,7 +6889,7 @@
       <c r="O148"/>
       <c r="P148"/>
     </row>
-    <row r="149" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="15"/>
@@ -6904,7 +6904,7 @@
       <c r="O149"/>
       <c r="P149"/>
     </row>
-    <row r="150" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="150" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="15"/>
@@ -6919,7 +6919,7 @@
       <c r="O150"/>
       <c r="P150"/>
     </row>
-    <row r="151" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="151" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="15"/>

</xml_diff>

<commit_message>
Herstel xlsx: niet bedoeld bij workflow-commit
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/sterkteberekingen funderingswapening Romfix (1).xlsx
+++ b/sterkteberekingen funderingswapening Romfix (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yenlo-my.sharepoint.com/personal/berntjan_bosma_yenlo_com/Documents/Bureaublad/Romfix/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3b3ce9f62cacfa1d/Romfix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{4343CC2F-9073-4518-94E3-F3DA523D61FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{800AA4D0-F76F-4907-8B03-D252897EA3DD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4343CC2F-9073-4518-94E3-F3DA523D61FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="791" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" tabRatio="791" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capping_Romfix" sheetId="115" r:id="rId1"/>
@@ -868,24 +868,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q151"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="3" width="13.140625" style="16" customWidth="1"/>
-    <col min="4" max="4" width="13" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="16" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" style="15" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.85546875" style="15" customWidth="1"/>
+    <col min="2" max="3" width="13.19921875" style="16" customWidth="1"/>
+    <col min="4" max="4" width="13.06640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.19921875" style="16" customWidth="1"/>
+    <col min="6" max="6" width="13.19921875" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.796875" style="15" customWidth="1"/>
+    <col min="9" max="9" width="11.19921875" style="15" customWidth="1"/>
+    <col min="10" max="10" width="10.796875" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.796875" style="15" customWidth="1"/>
     <col min="13" max="13" width="26" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.7109375" style="16"/>
+    <col min="14" max="15" width="10.796875" style="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.73046875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
         <v>49</v>
       </c>
@@ -906,7 +906,7 @@
       <c r="P1" s="12"/>
       <c r="Q1" s="14"/>
     </row>
-    <row r="2" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
@@ -924,7 +924,7 @@
       <c r="P2" s="12"/>
       <c r="Q2" s="14"/>
     </row>
-    <row r="3" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A3" s="11" t="s">
         <v>29</v>
       </c>
@@ -941,7 +941,7 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
@@ -956,7 +956,7 @@
       <c r="O4"/>
       <c r="P4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
         <v>30</v>
       </c>
@@ -977,7 +977,7 @@
       <c r="O5"/>
       <c r="P5"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" s="17" t="s">
         <v>36</v>
       </c>
@@ -998,7 +998,7 @@
       <c r="O6"/>
       <c r="P6"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
         <v>37</v>
       </c>
@@ -1019,7 +1019,7 @@
       <c r="O7"/>
       <c r="P7"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
         <v>38</v>
       </c>
@@ -1040,7 +1040,7 @@
       <c r="O8"/>
       <c r="P8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
@@ -1055,7 +1055,7 @@
       <c r="O9"/>
       <c r="P9"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" s="18" t="s">
         <v>32</v>
       </c>
@@ -1073,7 +1073,7 @@
       <c r="O10"/>
       <c r="P10"/>
     </row>
-    <row r="11" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="39.4" x14ac:dyDescent="0.4">
       <c r="A11" s="19" t="s">
         <v>20</v>
       </c>
@@ -1098,7 +1098,7 @@
       <c r="O11"/>
       <c r="P11"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>53</v>
       </c>
@@ -1129,7 +1129,7 @@
       <c r="O12"/>
       <c r="P12"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>55</v>
       </c>
@@ -1162,7 +1162,7 @@
       <c r="O13"/>
       <c r="P13"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>55</v>
       </c>
@@ -1191,7 +1191,7 @@
       <c r="O14"/>
       <c r="P14"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>7</v>
       </c>
@@ -1222,7 +1222,7 @@
       <c r="O15"/>
       <c r="P15"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -1234,7 +1234,7 @@
       <c r="O16"/>
       <c r="P16"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
         <v>33</v>
       </c>
@@ -1252,7 +1252,7 @@
       <c r="O17"/>
       <c r="P17"/>
     </row>
-    <row r="18" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="39.4" x14ac:dyDescent="0.4">
       <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
@@ -1277,7 +1277,7 @@
       <c r="O18"/>
       <c r="P18"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="str">
         <f>CONCATENATE("Wapening ",A13)</f>
         <v>Wapening Series 600 6F2 + R'cel + E'grid</v>
@@ -1304,7 +1304,7 @@
       <c r="O19"/>
       <c r="P19"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="str">
         <f>CONCATENATE("Wapening ",A14)</f>
         <v>Wapening Series 600 6F2 + R'cel + E'grid</v>
@@ -1331,7 +1331,7 @@
       <c r="O20"/>
       <c r="P20"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -1343,7 +1343,7 @@
       <c r="O21"/>
       <c r="P21"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="s">
         <v>27</v>
       </c>
@@ -1362,7 +1362,7 @@
       <c r="O22"/>
       <c r="P22"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A23" s="19" t="s">
         <v>20</v>
       </c>
@@ -1388,7 +1388,7 @@
       <c r="O23"/>
       <c r="P23"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="str">
         <f>A12</f>
         <v>Beton + fundering + series 800</v>
@@ -1418,7 +1418,7 @@
       <c r="O24"/>
       <c r="P24"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A25" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog</v>
@@ -1449,7 +1449,7 @@
       <c r="O25"/>
       <c r="P25"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend</v>
@@ -1477,7 +1477,7 @@
       <c r="O26"/>
       <c r="P26"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -1505,7 +1505,7 @@
       <c r="O27"/>
       <c r="P27"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A28" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog</v>
@@ -1536,7 +1536,7 @@
       <c r="O28"/>
       <c r="P28"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend</v>
@@ -1564,7 +1564,7 @@
       <c r="O29"/>
       <c r="P29"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -1592,7 +1592,7 @@
       <c r="O30"/>
       <c r="P30"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
         <v>7</v>
       </c>
@@ -1621,7 +1621,7 @@
       <c r="O31"/>
       <c r="P31"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -1636,7 +1636,7 @@
       <c r="O32"/>
       <c r="P32"/>
     </row>
-    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="18" t="s">
         <v>25</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="I33" s="29"/>
       <c r="J33" s="29"/>
     </row>
-    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="s">
         <v>3</v>
       </c>
@@ -1662,7 +1662,7 @@
       <c r="I34" s="29"/>
       <c r="J34" s="29"/>
     </row>
-    <row r="35" spans="1:16" s="31" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" s="31" customFormat="1" ht="52.5" x14ac:dyDescent="0.4">
       <c r="A35" s="19" t="s">
         <v>24</v>
       </c>
@@ -1697,7 +1697,7 @@
       <c r="M35" s="30"/>
       <c r="N35" s="30"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>23</v>
       </c>
@@ -1734,7 +1734,7 @@
       <c r="O36"/>
       <c r="P36"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" s="32" t="s">
         <v>16</v>
       </c>
@@ -1771,7 +1771,7 @@
       <c r="O37"/>
       <c r="P37"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" s="17" t="s">
         <v>21</v>
       </c>
@@ -1808,7 +1808,7 @@
       <c r="O38"/>
       <c r="P38"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" s="17" t="s">
         <v>22</v>
       </c>
@@ -1845,7 +1845,7 @@
       <c r="O39"/>
       <c r="P39"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" s="17" t="s">
         <v>2</v>
       </c>
@@ -1882,7 +1882,7 @@
       <c r="O40"/>
       <c r="P40"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" s="34" t="s">
         <v>11</v>
       </c>
@@ -1919,7 +1919,7 @@
       <c r="O41"/>
       <c r="P41"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" s="34" t="s">
         <v>12</v>
       </c>
@@ -1956,7 +1956,7 @@
       <c r="O42"/>
       <c r="P42"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" s="34" t="s">
         <v>13</v>
       </c>
@@ -1993,7 +1993,7 @@
       <c r="O43"/>
       <c r="P43"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" s="34" t="s">
         <v>14</v>
       </c>
@@ -2030,7 +2030,7 @@
       <c r="O44"/>
       <c r="P44"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" s="34" t="s">
         <v>15</v>
       </c>
@@ -2067,7 +2067,7 @@
       <c r="O45"/>
       <c r="P45"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46" s="34" t="s">
         <v>10</v>
       </c>
@@ -2104,7 +2104,7 @@
       <c r="O46"/>
       <c r="P46"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="15"/>
@@ -2119,7 +2119,7 @@
       <c r="O47"/>
       <c r="P47"/>
     </row>
-    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="36" t="s">
         <v>26</v>
       </c>
@@ -2132,7 +2132,7 @@
       <c r="I48" s="29"/>
       <c r="J48" s="29"/>
     </row>
-    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="36" t="s">
         <v>46</v>
       </c>
@@ -2145,7 +2145,7 @@
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A50" s="37" t="s">
         <v>20</v>
       </c>
@@ -2169,7 +2169,7 @@
       <c r="O50"/>
       <c r="P50"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2197,7 +2197,7 @@
       <c r="O51"/>
       <c r="P51"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2225,7 +2225,7 @@
       <c r="O52"/>
       <c r="P52"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2253,7 +2253,7 @@
       <c r="O53"/>
       <c r="P53"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2281,7 +2281,7 @@
       <c r="O54"/>
       <c r="P54"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2309,7 +2309,7 @@
       <c r="O55"/>
       <c r="P55"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2337,7 +2337,7 @@
       <c r="O56"/>
       <c r="P56"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
@@ -2352,7 +2352,7 @@
       <c r="O57"/>
       <c r="P57"/>
     </row>
-    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="s">
         <v>28</v>
       </c>
@@ -2365,7 +2365,7 @@
       <c r="I58" s="29"/>
       <c r="J58" s="29"/>
     </row>
-    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="s">
         <v>31</v>
       </c>
@@ -2378,7 +2378,7 @@
       <c r="I59" s="29"/>
       <c r="J59" s="29"/>
     </row>
-    <row r="60" spans="1:16" s="31" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" s="31" customFormat="1" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A60" s="19" t="s">
         <v>20</v>
       </c>
@@ -2401,7 +2401,7 @@
       <c r="J60" s="30"/>
       <c r="K60" s="30"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A61" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2433,7 +2433,7 @@
       <c r="O61"/>
       <c r="P61"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2465,7 +2465,7 @@
       <c r="O62"/>
       <c r="P62"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2497,7 +2497,7 @@
       <c r="O63"/>
       <c r="P63"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -2529,7 +2529,7 @@
       <c r="O64"/>
       <c r="P64"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid gewapend en dieper</v>
@@ -2561,7 +2561,7 @@
       <c r="O65"/>
       <c r="P65"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 600 6F2 + R'cel + E'grid ongewapend laag</v>
@@ -2593,7 +2593,7 @@
       <c r="O66"/>
       <c r="P66"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="17" t="str">
         <f>CONCATENATE(A$14," volledig ongewapend en dieper")</f>
         <v>Series 600 6F2 + R'cel + E'grid volledig ongewapend en dieper</v>
@@ -2625,7 +2625,7 @@
       <c r="O67"/>
       <c r="P67"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="15"/>
@@ -2640,7 +2640,7 @@
       <c r="O68"/>
       <c r="P68"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="15"/>
@@ -2655,7 +2655,7 @@
       <c r="O69"/>
       <c r="P69"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="15"/>
@@ -2670,7 +2670,7 @@
       <c r="O70"/>
       <c r="P70"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="15"/>
@@ -2685,7 +2685,7 @@
       <c r="O71"/>
       <c r="P71"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="15"/>
@@ -2700,7 +2700,7 @@
       <c r="O72"/>
       <c r="P72"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="15"/>
@@ -2715,7 +2715,7 @@
       <c r="O73"/>
       <c r="P73"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="15"/>
@@ -2730,7 +2730,7 @@
       <c r="O74"/>
       <c r="P74"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="15"/>
@@ -2745,7 +2745,7 @@
       <c r="O75"/>
       <c r="P75"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="15"/>
@@ -2760,7 +2760,7 @@
       <c r="O76"/>
       <c r="P76"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="15"/>
@@ -2775,7 +2775,7 @@
       <c r="O77"/>
       <c r="P77"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="15"/>
@@ -2790,7 +2790,7 @@
       <c r="O78"/>
       <c r="P78"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="15"/>
@@ -2805,7 +2805,7 @@
       <c r="O79"/>
       <c r="P79"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="15"/>
@@ -2820,7 +2820,7 @@
       <c r="O80"/>
       <c r="P80"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="15"/>
@@ -2835,7 +2835,7 @@
       <c r="O81"/>
       <c r="P81"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="15"/>
@@ -2850,7 +2850,7 @@
       <c r="O82"/>
       <c r="P82"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="15"/>
@@ -2865,7 +2865,7 @@
       <c r="O83"/>
       <c r="P83"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="15"/>
@@ -2880,7 +2880,7 @@
       <c r="O84"/>
       <c r="P84"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="15"/>
@@ -2895,7 +2895,7 @@
       <c r="O85"/>
       <c r="P85"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="15"/>
@@ -2910,7 +2910,7 @@
       <c r="O86"/>
       <c r="P86"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="15"/>
@@ -2925,7 +2925,7 @@
       <c r="O87"/>
       <c r="P87"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="15"/>
@@ -2940,7 +2940,7 @@
       <c r="O88"/>
       <c r="P88"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
@@ -2955,7 +2955,7 @@
       <c r="O89"/>
       <c r="P89"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="15"/>
@@ -2970,7 +2970,7 @@
       <c r="O90"/>
       <c r="P90"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="15"/>
@@ -2985,7 +2985,7 @@
       <c r="O91"/>
       <c r="P91"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="15"/>
@@ -3000,7 +3000,7 @@
       <c r="O92"/>
       <c r="P92"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="15"/>
@@ -3015,7 +3015,7 @@
       <c r="O93"/>
       <c r="P93"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="15"/>
@@ -3030,7 +3030,7 @@
       <c r="O94"/>
       <c r="P94"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="15"/>
@@ -3045,7 +3045,7 @@
       <c r="O95"/>
       <c r="P95"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="15"/>
@@ -3060,7 +3060,7 @@
       <c r="O96"/>
       <c r="P96"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -3075,7 +3075,7 @@
       <c r="O97"/>
       <c r="P97"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -3090,7 +3090,7 @@
       <c r="O98"/>
       <c r="P98"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -3105,7 +3105,7 @@
       <c r="O99"/>
       <c r="P99"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="15"/>
@@ -3120,7 +3120,7 @@
       <c r="O100"/>
       <c r="P100"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="15"/>
@@ -3135,7 +3135,7 @@
       <c r="O101"/>
       <c r="P101"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="15"/>
@@ -3150,7 +3150,7 @@
       <c r="O102"/>
       <c r="P102"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="15"/>
@@ -3165,7 +3165,7 @@
       <c r="O103"/>
       <c r="P103"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="15"/>
@@ -3180,7 +3180,7 @@
       <c r="O104"/>
       <c r="P104"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="15"/>
@@ -3195,7 +3195,7 @@
       <c r="O105"/>
       <c r="P105"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="15"/>
@@ -3210,7 +3210,7 @@
       <c r="O106"/>
       <c r="P106"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="15"/>
@@ -3225,7 +3225,7 @@
       <c r="O107"/>
       <c r="P107"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="15"/>
@@ -3240,7 +3240,7 @@
       <c r="O108"/>
       <c r="P108"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="15"/>
@@ -3255,7 +3255,7 @@
       <c r="O109"/>
       <c r="P109"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="15"/>
@@ -3270,7 +3270,7 @@
       <c r="O110"/>
       <c r="P110"/>
     </row>
-    <row r="111" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="15"/>
@@ -3285,7 +3285,7 @@
       <c r="O111"/>
       <c r="P111"/>
     </row>
-    <row r="112" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3300,7 +3300,7 @@
       <c r="O112"/>
       <c r="P112"/>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3315,7 +3315,7 @@
       <c r="O113"/>
       <c r="P113"/>
     </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -3330,7 +3330,7 @@
       <c r="O114"/>
       <c r="P114"/>
     </row>
-    <row r="115" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -3345,7 +3345,7 @@
       <c r="O115"/>
       <c r="P115"/>
     </row>
-    <row r="116" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -3360,7 +3360,7 @@
       <c r="O116"/>
       <c r="P116"/>
     </row>
-    <row r="117" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="15"/>
@@ -3375,7 +3375,7 @@
       <c r="O117"/>
       <c r="P117"/>
     </row>
-    <row r="118" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="15"/>
@@ -3390,7 +3390,7 @@
       <c r="O118"/>
       <c r="P118"/>
     </row>
-    <row r="119" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="15"/>
@@ -3405,7 +3405,7 @@
       <c r="O119"/>
       <c r="P119"/>
     </row>
-    <row r="120" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="15"/>
@@ -3420,7 +3420,7 @@
       <c r="O120"/>
       <c r="P120"/>
     </row>
-    <row r="121" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="15"/>
@@ -3435,7 +3435,7 @@
       <c r="O121"/>
       <c r="P121"/>
     </row>
-    <row r="122" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="15"/>
@@ -3450,7 +3450,7 @@
       <c r="O122"/>
       <c r="P122"/>
     </row>
-    <row r="123" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="15"/>
@@ -3465,7 +3465,7 @@
       <c r="O123"/>
       <c r="P123"/>
     </row>
-    <row r="124" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="15"/>
@@ -3480,7 +3480,7 @@
       <c r="O124"/>
       <c r="P124"/>
     </row>
-    <row r="125" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
@@ -3495,7 +3495,7 @@
       <c r="O125"/>
       <c r="P125"/>
     </row>
-    <row r="126" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -3510,7 +3510,7 @@
       <c r="O126"/>
       <c r="P126"/>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3525,7 +3525,7 @@
       <c r="O127"/>
       <c r="P127"/>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3540,7 +3540,7 @@
       <c r="O128"/>
       <c r="P128"/>
     </row>
-    <row r="129" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -3555,7 +3555,7 @@
       <c r="O129"/>
       <c r="P129"/>
     </row>
-    <row r="130" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -3570,7 +3570,7 @@
       <c r="O130"/>
       <c r="P130"/>
     </row>
-    <row r="131" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
@@ -3585,7 +3585,7 @@
       <c r="O131"/>
       <c r="P131"/>
     </row>
-    <row r="132" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="15"/>
@@ -3600,7 +3600,7 @@
       <c r="O132"/>
       <c r="P132"/>
     </row>
-    <row r="133" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="15"/>
@@ -3615,7 +3615,7 @@
       <c r="O133"/>
       <c r="P133"/>
     </row>
-    <row r="134" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="15"/>
@@ -3630,7 +3630,7 @@
       <c r="O134"/>
       <c r="P134"/>
     </row>
-    <row r="135" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="15"/>
@@ -3645,7 +3645,7 @@
       <c r="O135"/>
       <c r="P135"/>
     </row>
-    <row r="136" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="15"/>
@@ -3660,7 +3660,7 @@
       <c r="O136"/>
       <c r="P136"/>
     </row>
-    <row r="137" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="15"/>
@@ -3675,7 +3675,7 @@
       <c r="O137"/>
       <c r="P137"/>
     </row>
-    <row r="138" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -3690,7 +3690,7 @@
       <c r="O138"/>
       <c r="P138"/>
     </row>
-    <row r="139" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -3705,7 +3705,7 @@
       <c r="O139"/>
       <c r="P139"/>
     </row>
-    <row r="140" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
@@ -3720,7 +3720,7 @@
       <c r="O140"/>
       <c r="P140"/>
     </row>
-    <row r="141" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -3735,7 +3735,7 @@
       <c r="O141"/>
       <c r="P141"/>
     </row>
-    <row r="142" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -3750,7 +3750,7 @@
       <c r="O142"/>
       <c r="P142"/>
     </row>
-    <row r="143" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -3765,7 +3765,7 @@
       <c r="O143"/>
       <c r="P143"/>
     </row>
-    <row r="144" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -3780,7 +3780,7 @@
       <c r="O144"/>
       <c r="P144"/>
     </row>
-    <row r="145" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
@@ -3795,7 +3795,7 @@
       <c r="O145"/>
       <c r="P145"/>
     </row>
-    <row r="146" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="15"/>
@@ -3810,7 +3810,7 @@
       <c r="O146"/>
       <c r="P146"/>
     </row>
-    <row r="147" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="15"/>
@@ -3825,7 +3825,7 @@
       <c r="O147"/>
       <c r="P147"/>
     </row>
-    <row r="148" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="15"/>
@@ -3840,7 +3840,7 @@
       <c r="O148"/>
       <c r="P148"/>
     </row>
-    <row r="149" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="15"/>
@@ -3855,7 +3855,7 @@
       <c r="O149"/>
       <c r="P149"/>
     </row>
-    <row r="150" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="15"/>
@@ -3870,7 +3870,7 @@
       <c r="O150"/>
       <c r="P150"/>
     </row>
-    <row r="151" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="15"/>
@@ -3917,24 +3917,24 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q151"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="3" width="13.140625" style="16" customWidth="1"/>
-    <col min="4" max="4" width="13" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="16" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" style="15" customWidth="1"/>
-    <col min="10" max="10" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.85546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="44.06640625" customWidth="1"/>
+    <col min="2" max="3" width="13.19921875" style="16" customWidth="1"/>
+    <col min="4" max="4" width="13.06640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.19921875" style="16" customWidth="1"/>
+    <col min="6" max="6" width="13.19921875" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="11.796875" style="15" customWidth="1"/>
+    <col min="9" max="9" width="11.19921875" style="15" customWidth="1"/>
+    <col min="10" max="10" width="10.796875" style="15" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.796875" style="15" customWidth="1"/>
     <col min="13" max="13" width="26" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.7109375" style="16"/>
+    <col min="14" max="15" width="10.796875" style="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.73046875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
         <v>49</v>
       </c>
@@ -3955,7 +3955,7 @@
       <c r="P1" s="12"/>
       <c r="Q1" s="14"/>
     </row>
-    <row r="2" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
@@ -3973,7 +3973,7 @@
       <c r="P2" s="12"/>
       <c r="Q2" s="14"/>
     </row>
-    <row r="3" spans="1:17" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.4">
       <c r="A3" s="11" t="s">
         <v>29</v>
       </c>
@@ -3990,7 +3990,7 @@
       <c r="O3" s="12"/>
       <c r="P3" s="12"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
@@ -4005,7 +4005,7 @@
       <c r="O4"/>
       <c r="P4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
         <v>30</v>
       </c>
@@ -4026,7 +4026,7 @@
       <c r="O5"/>
       <c r="P5"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" s="17" t="s">
         <v>36</v>
       </c>
@@ -4047,7 +4047,7 @@
       <c r="O6"/>
       <c r="P6"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
         <v>37</v>
       </c>
@@ -4068,7 +4068,7 @@
       <c r="O7"/>
       <c r="P7"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
         <v>38</v>
       </c>
@@ -4089,7 +4089,7 @@
       <c r="O8"/>
       <c r="P8"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15"/>
@@ -4104,7 +4104,7 @@
       <c r="O9"/>
       <c r="P9"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" s="18" t="s">
         <v>32</v>
       </c>
@@ -4122,7 +4122,7 @@
       <c r="O10"/>
       <c r="P10"/>
     </row>
-    <row r="11" spans="1:17" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="39.4" x14ac:dyDescent="0.4">
       <c r="A11" s="19" t="s">
         <v>20</v>
       </c>
@@ -4147,7 +4147,7 @@
       <c r="O11"/>
       <c r="P11"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>52</v>
       </c>
@@ -4178,7 +4178,7 @@
       <c r="O12"/>
       <c r="P12"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -4186,15 +4186,15 @@
         <v>250</v>
       </c>
       <c r="C13" s="2">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="D13" s="9">
         <f>IF(F13="vast",C13,IF(F13="vrij",G46,""))</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E13" s="5">
         <f>IF(F13="vrij",E25,IF(F13="vast",MAX(D13,E25),""))</f>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>51</v>
@@ -4211,7 +4211,7 @@
       <c r="O13"/>
       <c r="P13"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>56</v>
       </c>
@@ -4240,7 +4240,7 @@
       <c r="O14"/>
       <c r="P14"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>7</v>
       </c>
@@ -4271,7 +4271,7 @@
       <c r="O15"/>
       <c r="P15"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
@@ -4283,7 +4283,7 @@
       <c r="O16"/>
       <c r="P16"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
         <v>33</v>
       </c>
@@ -4301,7 +4301,7 @@
       <c r="O17"/>
       <c r="P17"/>
     </row>
-    <row r="18" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="39.4" x14ac:dyDescent="0.4">
       <c r="A18" s="19" t="s">
         <v>20</v>
       </c>
@@ -4326,7 +4326,7 @@
       <c r="O18"/>
       <c r="P18"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="str">
         <f>CONCATENATE("Wapening ",A13)</f>
         <v>Wapening Series 800 Type 1 + R'cel + E'grid</v>
@@ -4353,7 +4353,7 @@
       <c r="O19"/>
       <c r="P19"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="str">
         <f>CONCATENATE("Wapening ",A14)</f>
         <v>Wapening Series 800 Type 1 + R'cel + E'grid</v>
@@ -4380,7 +4380,7 @@
       <c r="O20"/>
       <c r="P20"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
@@ -4392,7 +4392,7 @@
       <c r="O21"/>
       <c r="P21"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="s">
         <v>27</v>
       </c>
@@ -4411,7 +4411,7 @@
       <c r="O22"/>
       <c r="P22"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A23" s="19" t="s">
         <v>20</v>
       </c>
@@ -4437,7 +4437,7 @@
       <c r="O23"/>
       <c r="P23"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="str">
         <f>A12</f>
         <v>Beton + fundering</v>
@@ -4467,7 +4467,7 @@
       <c r="O24"/>
       <c r="P24"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A25" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog</v>
@@ -4482,11 +4482,11 @@
       </c>
       <c r="D25" s="22">
         <f>IF(B25=0,D26,ROUND(D28/F61,0))</f>
-        <v>282</v>
+        <v>381</v>
       </c>
       <c r="E25" s="23">
         <f>D51</f>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="F25" s="24"/>
       <c r="H25"/>
@@ -4498,7 +4498,7 @@
       <c r="O25"/>
       <c r="P25"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend</v>
@@ -4509,11 +4509,11 @@
       </c>
       <c r="C26" s="5">
         <f>IF(B26=0,0,ROUND(MIN(D19*D27,E19*C13),0))</f>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="D26" s="5">
         <f>IF(B26=0,D27,ROUND(D28/F62,0))</f>
-        <v>282</v>
+        <v>381</v>
       </c>
       <c r="E26" s="25"/>
       <c r="F26" s="24"/>
@@ -4526,7 +4526,7 @@
       <c r="O26"/>
       <c r="P26"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -4554,7 +4554,7 @@
       <c r="O27"/>
       <c r="P27"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A28" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog</v>
@@ -4585,7 +4585,7 @@
       <c r="O28"/>
       <c r="P28"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend</v>
@@ -4613,7 +4613,7 @@
       <c r="O29"/>
       <c r="P29"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -4641,7 +4641,7 @@
       <c r="O30"/>
       <c r="P30"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
         <v>7</v>
       </c>
@@ -4670,7 +4670,7 @@
       <c r="O31"/>
       <c r="P31"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -4685,7 +4685,7 @@
       <c r="O32"/>
       <c r="P32"/>
     </row>
-    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="18" t="s">
         <v>25</v>
       </c>
@@ -4698,7 +4698,7 @@
       <c r="I33" s="29"/>
       <c r="J33" s="29"/>
     </row>
-    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="s">
         <v>3</v>
       </c>
@@ -4711,7 +4711,7 @@
       <c r="I34" s="29"/>
       <c r="J34" s="29"/>
     </row>
-    <row r="35" spans="1:16" s="31" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" s="31" customFormat="1" ht="52.5" x14ac:dyDescent="0.4">
       <c r="A35" s="19" t="s">
         <v>24</v>
       </c>
@@ -4746,7 +4746,7 @@
       <c r="M35" s="30"/>
       <c r="N35" s="30"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>23</v>
       </c>
@@ -4783,7 +4783,7 @@
       <c r="O36"/>
       <c r="P36"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A37" s="32" t="s">
         <v>16</v>
       </c>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="E37" s="23">
         <f>D26</f>
-        <v>282</v>
+        <v>381</v>
       </c>
       <c r="F37" s="5">
         <f>C15</f>
@@ -4820,7 +4820,7 @@
       <c r="O37"/>
       <c r="P37"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A38" s="17" t="s">
         <v>21</v>
       </c>
@@ -4834,11 +4834,11 @@
       </c>
       <c r="D38" s="5">
         <f>C13</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E38" s="5">
         <f>C13</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F38" s="5">
         <f>C14</f>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="G38" s="5">
         <f>C13</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H38" s="16"/>
       <c r="I38" s="16"/>
@@ -4857,7 +4857,7 @@
       <c r="O38"/>
       <c r="P38"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A39" s="17" t="s">
         <v>22</v>
       </c>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="E39" s="6">
         <f t="shared" si="0"/>
-        <v>282</v>
+        <v>381</v>
       </c>
       <c r="F39" s="6">
         <f t="shared" si="0"/>
@@ -4894,7 +4894,7 @@
       <c r="O39"/>
       <c r="P39"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A40" s="17" t="s">
         <v>2</v>
       </c>
@@ -4931,7 +4931,7 @@
       <c r="O40"/>
       <c r="P40"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A41" s="34" t="s">
         <v>11</v>
       </c>
@@ -4945,11 +4945,11 @@
       </c>
       <c r="D41" s="35">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E41" s="35">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F41" s="35">
         <f t="shared" si="2"/>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="G41" s="35">
         <f t="shared" si="2"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H41" s="16"/>
       <c r="I41" s="16"/>
@@ -4968,7 +4968,7 @@
       <c r="O41"/>
       <c r="P41"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A42" s="34" t="s">
         <v>12</v>
       </c>
@@ -4982,11 +4982,11 @@
       </c>
       <c r="D42" s="35">
         <f t="shared" si="3"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E42" s="35">
         <f t="shared" si="3"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F42" s="35">
         <f t="shared" si="3"/>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="G42" s="35">
         <f t="shared" si="3"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H42" s="16"/>
       <c r="I42" s="16"/>
@@ -5005,7 +5005,7 @@
       <c r="O42"/>
       <c r="P42"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A43" s="34" t="s">
         <v>13</v>
       </c>
@@ -5019,11 +5019,11 @@
       </c>
       <c r="D43" s="35">
         <f t="shared" si="4"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E43" s="35">
         <f t="shared" si="4"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F43" s="35">
         <f t="shared" si="4"/>
@@ -5031,7 +5031,7 @@
       </c>
       <c r="G43" s="35">
         <f t="shared" si="4"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H43" s="16"/>
       <c r="I43" s="16"/>
@@ -5042,7 +5042,7 @@
       <c r="O43"/>
       <c r="P43"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A44" s="34" t="s">
         <v>14</v>
       </c>
@@ -5056,11 +5056,11 @@
       </c>
       <c r="D44" s="35">
         <f t="shared" si="5"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E44" s="35">
         <f t="shared" si="5"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F44" s="35">
         <f t="shared" si="5"/>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="G44" s="35">
         <f t="shared" si="5"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H44" s="16"/>
       <c r="I44" s="16"/>
@@ -5079,7 +5079,7 @@
       <c r="O44"/>
       <c r="P44"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A45" s="34" t="s">
         <v>15</v>
       </c>
@@ -5093,11 +5093,11 @@
       </c>
       <c r="D45" s="35">
         <f t="shared" ref="D45:E45" si="6">MIN(D40*D37,D38)</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E45" s="35">
         <f t="shared" si="6"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F45" s="35">
         <f>MIN(F40*F37,F38)</f>
@@ -5105,7 +5105,7 @@
       </c>
       <c r="G45" s="35">
         <f>MIN(G40*G37,G38)</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H45" s="16"/>
       <c r="I45" s="16"/>
@@ -5116,7 +5116,7 @@
       <c r="O45"/>
       <c r="P45"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A46" s="34" t="s">
         <v>10</v>
       </c>
@@ -5130,11 +5130,11 @@
       </c>
       <c r="D46" s="35">
         <f t="shared" si="7"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E46" s="35">
         <f t="shared" si="7"/>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F46" s="35">
         <f>ROUND(AVERAGE(F41:F45),0)</f>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="G46" s="35">
         <f>ROUND(AVERAGE(G41:G45),0)</f>
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="H46" s="16"/>
       <c r="I46" s="16"/>
@@ -5153,7 +5153,7 @@
       <c r="O46"/>
       <c r="P46"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="15"/>
@@ -5168,7 +5168,7 @@
       <c r="O47"/>
       <c r="P47"/>
     </row>
-    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="36" t="s">
         <v>26</v>
       </c>
@@ -5181,7 +5181,7 @@
       <c r="I48" s="29"/>
       <c r="J48" s="29"/>
     </row>
-    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="36" t="s">
         <v>46</v>
       </c>
@@ -5194,7 +5194,7 @@
       <c r="I49" s="29"/>
       <c r="J49" s="29"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A50" s="37" t="s">
         <v>20</v>
       </c>
@@ -5218,7 +5218,7 @@
       <c r="O50"/>
       <c r="P50"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5233,7 +5233,7 @@
       </c>
       <c r="D51" s="5">
         <f>ROUND(((B51*C51^(1/3)+B52*C52^(1/3)+B53*C53^(1/3))/(B51+B52+B53))^3,0)</f>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="E51" s="15"/>
       <c r="F51" s="15"/>
@@ -5246,7 +5246,7 @@
       <c r="O51"/>
       <c r="P51"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5257,11 +5257,11 @@
       </c>
       <c r="C52" s="38">
         <f t="shared" si="9"/>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="D52" s="5">
         <f>IF(B52+B53=0,0,IF(B53=0,C52,ROUND(((B52*C52^(1/3)+B53*C53^(1/3))/(B52+B53))^3,0)))</f>
-        <v>344</v>
+        <v>645</v>
       </c>
       <c r="E52" s="15"/>
       <c r="F52" s="15"/>
@@ -5274,7 +5274,7 @@
       <c r="O52"/>
       <c r="P52"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5302,7 +5302,7 @@
       <c r="O53"/>
       <c r="P53"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5330,7 +5330,7 @@
       <c r="O54"/>
       <c r="P54"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5358,7 +5358,7 @@
       <c r="O55"/>
       <c r="P55"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5386,7 +5386,7 @@
       <c r="O56"/>
       <c r="P56"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="15"/>
@@ -5401,7 +5401,7 @@
       <c r="O57"/>
       <c r="P57"/>
     </row>
-    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="18" t="s">
         <v>28</v>
       </c>
@@ -5414,7 +5414,7 @@
       <c r="I58" s="29"/>
       <c r="J58" s="29"/>
     </row>
-    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="18" t="s">
         <v>31</v>
       </c>
@@ -5427,7 +5427,7 @@
       <c r="I59" s="29"/>
       <c r="J59" s="29"/>
     </row>
-    <row r="60" spans="1:16" s="31" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:16" s="31" customFormat="1" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A60" s="19" t="s">
         <v>20</v>
       </c>
@@ -5450,7 +5450,7 @@
       <c r="J60" s="30"/>
       <c r="K60" s="30"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A61" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5468,11 +5468,11 @@
       </c>
       <c r="E61" s="40">
         <f>D51/D28</f>
-        <v>1.4700854700854702</v>
+        <v>2.7564102564102564</v>
       </c>
       <c r="F61" s="40">
         <f>IF(D61="","",(B61/SQRT(B61^2+C61^2*E61^(2/3)))*(1-1/E61)+1/E61)</f>
-        <v>0.82946507354766585</v>
+        <v>0.61348089534453298</v>
       </c>
       <c r="H61"/>
       <c r="J61" s="16"/>
@@ -5482,7 +5482,7 @@
       <c r="O61"/>
       <c r="P61"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" s="17" t="str">
         <f>CONCATENATE(A$13," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5500,11 +5500,11 @@
       </c>
       <c r="E62" s="40">
         <f>D52/D28</f>
-        <v>1.4700854700854702</v>
+        <v>2.7564102564102564</v>
       </c>
       <c r="F62" s="40">
         <f t="shared" ref="F62:F67" si="11">IF(D62="","",(B62/SQRT(B62^2+C62^2*E62^(2/3)))*(1-1/E62)+1/E62)</f>
-        <v>0.82946507354766585</v>
+        <v>0.61348089534453298</v>
       </c>
       <c r="H62"/>
       <c r="J62" s="16"/>
@@ -5514,7 +5514,7 @@
       <c r="O62"/>
       <c r="P62"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63" s="17" t="str">
         <f>CONCATENATE(A$13," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5546,7 +5546,7 @@
       <c r="O63"/>
       <c r="P63"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend hoog en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend hoog en dieper</v>
@@ -5578,7 +5578,7 @@
       <c r="O64"/>
       <c r="P64"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A65" s="17" t="str">
         <f>CONCATENATE(A$14," gewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid gewapend en dieper</v>
@@ -5610,7 +5610,7 @@
       <c r="O65"/>
       <c r="P65"/>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A66" s="17" t="str">
         <f>CONCATENATE(A$14," ongewapend laag")</f>
         <v>Series 800 Type 1 + R'cel + E'grid ongewapend laag</v>
@@ -5642,7 +5642,7 @@
       <c r="O66"/>
       <c r="P66"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A67" s="17" t="str">
         <f>CONCATENATE(A$14," volledig ongewapend en dieper")</f>
         <v>Series 800 Type 1 + R'cel + E'grid volledig ongewapend en dieper</v>
@@ -5674,7 +5674,7 @@
       <c r="O67"/>
       <c r="P67"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="15"/>
@@ -5689,7 +5689,7 @@
       <c r="O68"/>
       <c r="P68"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="15"/>
@@ -5704,7 +5704,7 @@
       <c r="O69"/>
       <c r="P69"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="15"/>
@@ -5719,7 +5719,7 @@
       <c r="O70"/>
       <c r="P70"/>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="15"/>
@@ -5734,7 +5734,7 @@
       <c r="O71"/>
       <c r="P71"/>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="15"/>
@@ -5749,7 +5749,7 @@
       <c r="O72"/>
       <c r="P72"/>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="15"/>
@@ -5764,7 +5764,7 @@
       <c r="O73"/>
       <c r="P73"/>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="15"/>
@@ -5779,7 +5779,7 @@
       <c r="O74"/>
       <c r="P74"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="15"/>
@@ -5794,7 +5794,7 @@
       <c r="O75"/>
       <c r="P75"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="15"/>
@@ -5809,7 +5809,7 @@
       <c r="O76"/>
       <c r="P76"/>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="15"/>
@@ -5824,7 +5824,7 @@
       <c r="O77"/>
       <c r="P77"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="15"/>
@@ -5839,7 +5839,7 @@
       <c r="O78"/>
       <c r="P78"/>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="15"/>
@@ -5854,7 +5854,7 @@
       <c r="O79"/>
       <c r="P79"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="15"/>
@@ -5869,7 +5869,7 @@
       <c r="O80"/>
       <c r="P80"/>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="15"/>
@@ -5884,7 +5884,7 @@
       <c r="O81"/>
       <c r="P81"/>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="15"/>
@@ -5899,7 +5899,7 @@
       <c r="O82"/>
       <c r="P82"/>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="15"/>
@@ -5914,7 +5914,7 @@
       <c r="O83"/>
       <c r="P83"/>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="15"/>
@@ -5929,7 +5929,7 @@
       <c r="O84"/>
       <c r="P84"/>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="15"/>
@@ -5944,7 +5944,7 @@
       <c r="O85"/>
       <c r="P85"/>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="15"/>
@@ -5959,7 +5959,7 @@
       <c r="O86"/>
       <c r="P86"/>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="15"/>
@@ -5974,7 +5974,7 @@
       <c r="O87"/>
       <c r="P87"/>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="15"/>
@@ -5989,7 +5989,7 @@
       <c r="O88"/>
       <c r="P88"/>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="15"/>
@@ -6004,7 +6004,7 @@
       <c r="O89"/>
       <c r="P89"/>
     </row>
-    <row r="90" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="15"/>
@@ -6019,7 +6019,7 @@
       <c r="O90"/>
       <c r="P90"/>
     </row>
-    <row r="91" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="15"/>
@@ -6034,7 +6034,7 @@
       <c r="O91"/>
       <c r="P91"/>
     </row>
-    <row r="92" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="15"/>
@@ -6049,7 +6049,7 @@
       <c r="O92"/>
       <c r="P92"/>
     </row>
-    <row r="93" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="15"/>
@@ -6064,7 +6064,7 @@
       <c r="O93"/>
       <c r="P93"/>
     </row>
-    <row r="94" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="15"/>
@@ -6079,7 +6079,7 @@
       <c r="O94"/>
       <c r="P94"/>
     </row>
-    <row r="95" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="15"/>
@@ -6094,7 +6094,7 @@
       <c r="O95"/>
       <c r="P95"/>
     </row>
-    <row r="96" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="15"/>
@@ -6109,7 +6109,7 @@
       <c r="O96"/>
       <c r="P96"/>
     </row>
-    <row r="97" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -6124,7 +6124,7 @@
       <c r="O97"/>
       <c r="P97"/>
     </row>
-    <row r="98" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -6139,7 +6139,7 @@
       <c r="O98"/>
       <c r="P98"/>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -6154,7 +6154,7 @@
       <c r="O99"/>
       <c r="P99"/>
     </row>
-    <row r="100" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="15"/>
@@ -6169,7 +6169,7 @@
       <c r="O100"/>
       <c r="P100"/>
     </row>
-    <row r="101" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="15"/>
@@ -6184,7 +6184,7 @@
       <c r="O101"/>
       <c r="P101"/>
     </row>
-    <row r="102" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="15"/>
@@ -6199,7 +6199,7 @@
       <c r="O102"/>
       <c r="P102"/>
     </row>
-    <row r="103" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="15"/>
@@ -6214,7 +6214,7 @@
       <c r="O103"/>
       <c r="P103"/>
     </row>
-    <row r="104" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="15"/>
@@ -6229,7 +6229,7 @@
       <c r="O104"/>
       <c r="P104"/>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="15"/>
@@ -6244,7 +6244,7 @@
       <c r="O105"/>
       <c r="P105"/>
     </row>
-    <row r="106" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="15"/>
@@ -6259,7 +6259,7 @@
       <c r="O106"/>
       <c r="P106"/>
     </row>
-    <row r="107" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="15"/>
@@ -6274,7 +6274,7 @@
       <c r="O107"/>
       <c r="P107"/>
     </row>
-    <row r="108" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="15"/>
@@ -6289,7 +6289,7 @@
       <c r="O108"/>
       <c r="P108"/>
     </row>
-    <row r="109" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="15"/>
@@ -6304,7 +6304,7 @@
       <c r="O109"/>
       <c r="P109"/>
     </row>
-    <row r="110" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="15"/>
@@ -6319,7 +6319,7 @@
       <c r="O110"/>
       <c r="P110"/>
     </row>
-    <row r="111" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="15"/>
@@ -6334,7 +6334,7 @@
       <c r="O111"/>
       <c r="P111"/>
     </row>
-    <row r="112" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -6349,7 +6349,7 @@
       <c r="O112"/>
       <c r="P112"/>
     </row>
-    <row r="113" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -6364,7 +6364,7 @@
       <c r="O113"/>
       <c r="P113"/>
     </row>
-    <row r="114" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -6379,7 +6379,7 @@
       <c r="O114"/>
       <c r="P114"/>
     </row>
-    <row r="115" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -6394,7 +6394,7 @@
       <c r="O115"/>
       <c r="P115"/>
     </row>
-    <row r="116" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -6409,7 +6409,7 @@
       <c r="O116"/>
       <c r="P116"/>
     </row>
-    <row r="117" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="15"/>
@@ -6424,7 +6424,7 @@
       <c r="O117"/>
       <c r="P117"/>
     </row>
-    <row r="118" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="15"/>
@@ -6439,7 +6439,7 @@
       <c r="O118"/>
       <c r="P118"/>
     </row>
-    <row r="119" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="15"/>
@@ -6454,7 +6454,7 @@
       <c r="O119"/>
       <c r="P119"/>
     </row>
-    <row r="120" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="15"/>
@@ -6469,7 +6469,7 @@
       <c r="O120"/>
       <c r="P120"/>
     </row>
-    <row r="121" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="15"/>
@@ -6484,7 +6484,7 @@
       <c r="O121"/>
       <c r="P121"/>
     </row>
-    <row r="122" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="15"/>
@@ -6499,7 +6499,7 @@
       <c r="O122"/>
       <c r="P122"/>
     </row>
-    <row r="123" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="15"/>
@@ -6514,7 +6514,7 @@
       <c r="O123"/>
       <c r="P123"/>
     </row>
-    <row r="124" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="15"/>
@@ -6529,7 +6529,7 @@
       <c r="O124"/>
       <c r="P124"/>
     </row>
-    <row r="125" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
@@ -6544,7 +6544,7 @@
       <c r="O125"/>
       <c r="P125"/>
     </row>
-    <row r="126" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -6559,7 +6559,7 @@
       <c r="O126"/>
       <c r="P126"/>
     </row>
-    <row r="127" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -6574,7 +6574,7 @@
       <c r="O127"/>
       <c r="P127"/>
     </row>
-    <row r="128" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -6589,7 +6589,7 @@
       <c r="O128"/>
       <c r="P128"/>
     </row>
-    <row r="129" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -6604,7 +6604,7 @@
       <c r="O129"/>
       <c r="P129"/>
     </row>
-    <row r="130" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -6619,7 +6619,7 @@
       <c r="O130"/>
       <c r="P130"/>
     </row>
-    <row r="131" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
@@ -6634,7 +6634,7 @@
       <c r="O131"/>
       <c r="P131"/>
     </row>
-    <row r="132" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="15"/>
@@ -6649,7 +6649,7 @@
       <c r="O132"/>
       <c r="P132"/>
     </row>
-    <row r="133" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="15"/>
@@ -6664,7 +6664,7 @@
       <c r="O133"/>
       <c r="P133"/>
     </row>
-    <row r="134" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="15"/>
@@ -6679,7 +6679,7 @@
       <c r="O134"/>
       <c r="P134"/>
     </row>
-    <row r="135" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="15"/>
@@ -6694,7 +6694,7 @@
       <c r="O135"/>
       <c r="P135"/>
     </row>
-    <row r="136" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="15"/>
@@ -6709,7 +6709,7 @@
       <c r="O136"/>
       <c r="P136"/>
     </row>
-    <row r="137" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="15"/>
@@ -6724,7 +6724,7 @@
       <c r="O137"/>
       <c r="P137"/>
     </row>
-    <row r="138" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="15"/>
@@ -6739,7 +6739,7 @@
       <c r="O138"/>
       <c r="P138"/>
     </row>
-    <row r="139" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="15"/>
@@ -6754,7 +6754,7 @@
       <c r="O139"/>
       <c r="P139"/>
     </row>
-    <row r="140" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
@@ -6769,7 +6769,7 @@
       <c r="O140"/>
       <c r="P140"/>
     </row>
-    <row r="141" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -6784,7 +6784,7 @@
       <c r="O141"/>
       <c r="P141"/>
     </row>
-    <row r="142" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -6799,7 +6799,7 @@
       <c r="O142"/>
       <c r="P142"/>
     </row>
-    <row r="143" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -6814,7 +6814,7 @@
       <c r="O143"/>
       <c r="P143"/>
     </row>
-    <row r="144" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -6829,7 +6829,7 @@
       <c r="O144"/>
       <c r="P144"/>
     </row>
-    <row r="145" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
@@ -6844,7 +6844,7 @@
       <c r="O145"/>
       <c r="P145"/>
     </row>
-    <row r="146" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="15"/>
@@ -6859,7 +6859,7 @@
       <c r="O146"/>
       <c r="P146"/>
     </row>
-    <row r="147" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="15"/>
@@ -6874,7 +6874,7 @@
       <c r="O147"/>
       <c r="P147"/>
     </row>
-    <row r="148" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="15"/>
@@ -6889,7 +6889,7 @@
       <c r="O148"/>
       <c r="P148"/>
     </row>
-    <row r="149" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="15"/>
@@ -6904,7 +6904,7 @@
       <c r="O149"/>
       <c r="P149"/>
     </row>
-    <row r="150" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="15"/>
@@ -6919,7 +6919,7 @@
       <c r="O150"/>
       <c r="P150"/>
     </row>
-    <row r="151" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="15"/>

</xml_diff>